<commit_message>
Update supplementary title metadata
</commit_message>
<xml_diff>
--- a/supplementary/ESM_2.xlsx
+++ b/supplementary/ESM_2.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="R7472ecde4d70405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLENA Results" sheetId="2" r:id="Rb2bff09c957d4ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Rbb0ab25cfac64cad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="Rae3e4c3c2ec74491"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLENA Results" sheetId="2" r:id="Rea7d1693879f4943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R4435fec924c74dd6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -555,7 +555,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="92" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="78" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -572,12 +572,12 @@
         <x:v>Online Resource 2: PLENA Beta-Class Results Workbook</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="34" customHeight="1">
+    <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="20" t="str">
         <x:v>Article Title</x:v>
       </x:c>
       <x:c r="B3" s="21" t="str">
-        <x:v>High-Performance C++ Reimplementation and Optimization of the Gibbs' Model for Analyzing Structural Complexity in Urban Drainage Networks</x:v>
+        <x:v>City-Wide Assessment of Structural Complexity in Urban Drainage Networks Using Gibbs’ Model for Flood Risk Management</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -620,7 +620,7 @@
         <x:v>Online Resource 2</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="34" customHeight="1">
+    <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="20" t="str">
         <x:v>Caption</x:v>
       </x:c>
@@ -4017,7 +4017,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2712a61a3ed647e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c38ba93301e4825"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Remove internal QA traces from public supplements
</commit_message>
<xml_diff>
--- a/supplementary/ESM_2.xlsx
+++ b/supplementary/ESM_2.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="Rae3e4c3c2ec74491"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLENA Results" sheetId="2" r:id="Rea7d1693879f4943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="R4435fec924c74dd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metadata" sheetId="1" r:id="R90ed514c04754099"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLENA Results" sheetId="2" r:id="Rf8163ccac15e43cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" r:id="Ra0db590c93264039"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4017,7 +4017,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c38ba93301e4825"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd6ad6e10a56418c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4033,16 +4033,16 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>PLENA Results - English Workbook QA</x:v>
+        <x:v>PLENA Results - English Workbook Summary</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>PLENA Results - English Workbook QA</x:v>
+        <x:v>PLENA Results - English Workbook Summary</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>PLENA Results - English Workbook QA</x:v>
+        <x:v>PLENA Results - English Workbook Summary</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>PLENA Results - English Workbook QA</x:v>
+        <x:v>PLENA Results - English Workbook Summary</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1"/>
@@ -4063,7 +4063,7 @@
         <x:v>239</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="28" customHeight="1">
+    <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="36" t="str">
         <x:v>Main sheet columns</x:v>
       </x:c>
@@ -4071,7 +4071,7 @@
         <x:v>Catchment ID; Catchment Name; Kim et al., 2017; This Study</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="28" customHeight="1">
+    <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="36" t="str">
         <x:v>Main sheet order</x:v>
       </x:c>

</xml_diff>